<commit_message>
test: refresh APS spreadsheet fixtures
</commit_message>
<xml_diff>
--- a/test-data/3.多品共模.xlsx
+++ b/test-data/3.多品共模.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="28800" windowHeight="12255" activeTab="1"/>
+    <workbookView windowWidth="14280" windowHeight="13845"/>
   </bookViews>
   <sheets>
     <sheet name="共模规则" sheetId="1" r:id="rId1"/>
@@ -1216,7 +1216,6 @@
       <c r="B3" t="s">
         <v>8</v>
       </c>
-      <c r="C3"/>
       <c r="E3" t="s">
         <v>9</v>
       </c>
@@ -1228,7 +1227,6 @@
       <c r="B4" t="s">
         <v>11</v>
       </c>
-      <c r="C4"/>
       <c r="E4" t="s">
         <v>9</v>
       </c>
@@ -1240,7 +1238,6 @@
       <c r="B5" t="s">
         <v>13</v>
       </c>
-      <c r="C5"/>
       <c r="E5" t="s">
         <v>9</v>
       </c>
@@ -1252,7 +1249,6 @@
       <c r="B6" t="s">
         <v>15</v>
       </c>
-      <c r="C6"/>
       <c r="E6" t="s">
         <v>9</v>
       </c>
@@ -1264,7 +1260,6 @@
       <c r="B7" t="s">
         <v>17</v>
       </c>
-      <c r="C7"/>
       <c r="E7" t="s">
         <v>9</v>
       </c>
@@ -1276,7 +1271,6 @@
       <c r="B8" t="s">
         <v>19</v>
       </c>
-      <c r="C8"/>
       <c r="E8" t="s">
         <v>9</v>
       </c>
@@ -1288,7 +1282,6 @@
       <c r="B9" t="s">
         <v>21</v>
       </c>
-      <c r="C9"/>
       <c r="E9" t="s">
         <v>9</v>
       </c>
@@ -1300,7 +1293,6 @@
       <c r="B10" t="s">
         <v>23</v>
       </c>
-      <c r="C10"/>
       <c r="E10" t="s">
         <v>9</v>
       </c>
@@ -1312,7 +1304,6 @@
       <c r="B11" t="s">
         <v>25</v>
       </c>
-      <c r="C11"/>
       <c r="E11" t="s">
         <v>9</v>
       </c>

</xml_diff>